<commit_message>
preset tables in website
</commit_message>
<xml_diff>
--- a/data/exports/schemas/schema_1.13.1_dev.xlsx
+++ b/data/exports/schemas/schema_1.13.1_dev.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schneids\code\peexcel\data\exports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schneids\code\peexcel\data\exports\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1289C8B1-47FD-432F-AF97-ED18C9E391F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF5BA57E-B1D8-4C43-83D9-C47918DE1998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="23" activeTab="31" xr2:uid="{F7E5CCF4-99AF-4562-B3AA-2B99BA5C8B17}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="23" activeTab="31" xr2:uid="{BD89F594-14EF-4A5D-B864-24B378D385C0}"/>
   </bookViews>
   <sheets>
     <sheet name="META" sheetId="2" r:id="rId1"/>
@@ -15707,24 +15707,120 @@
     <t>Live</t>
   </si>
   <si>
+    <t xml:space="preserve">Neubau konventionell Stahlbeton </t>
+  </si>
+  <si>
+    <t>Bet</t>
+  </si>
+  <si>
+    <t>Passivhaus</t>
+  </si>
+  <si>
+    <t>AWm 01 a Stahlbeton-Außenwand, WDVS</t>
+  </si>
+  <si>
+    <t>DAm 03 a Stahlbeton-Flachdach als Warmdach</t>
+  </si>
+  <si>
+    <t>Efo 01 a Plattenfundament, oberseitig gedämmt, Nassestrich</t>
+  </si>
+  <si>
+    <t>GDm 01 a Stahlbeton-Geschoßdecke, Nassestrich (Nassräume)</t>
+  </si>
+  <si>
+    <t>DAm 06 a Stahlbeton-Flachdach mit Terrassenaufbau</t>
+  </si>
+  <si>
+    <t>KDu 01 a Kellerdecke massiv, unterseitig gedämmt</t>
+  </si>
+  <si>
+    <t>ADm 01 a Stahlbetondecke über Außenluft, Distanzboden</t>
+  </si>
+  <si>
+    <t>EAm 02 a Erdberührte Stahlbeton-Außenwand</t>
+  </si>
+  <si>
+    <t>IWl 01 a Ständer-Scheidewand, nichttragend</t>
+  </si>
+  <si>
+    <t>Neubau_Stb_IWm 05 a Schwere Hochlochziegel-Wohnungstrennwand</t>
+  </si>
+  <si>
+    <t>Erdberührte Wand Keller</t>
+  </si>
+  <si>
+    <t>1_UG_TG_BP_01d Bodenplatte STB 120 kg/m³ WU Beton bei drückendem Wasser, weiße Wanne, Asphaltbelag</t>
+  </si>
+  <si>
+    <t>1_UG_TG_Stü_01 Stützen</t>
+  </si>
+  <si>
+    <t>1_UG_TG_TW_01 Trennwand zu TG STB 100kg/m³ TG (tragend + Brandschutz)</t>
+  </si>
+  <si>
+    <t>Holz-Alu-Rahmen Fichte &gt;= 91 Stockrahmentiefe &lt; 109</t>
+  </si>
+  <si>
+    <t>Dreifach-Wärmeschutzglas, Argon, 40 &lt; Scheibenstärke</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>Zie</t>
+  </si>
+  <si>
+    <t>Neubau konventionell Ziegel</t>
+  </si>
+  <si>
+    <t>AWm 06 a Schwere Hochlochziegel-Außenwand, Spezial-WDVS</t>
+  </si>
+  <si>
+    <t>GDm 03 a Ziegel-Geschoßdecke ohne Aufbeton</t>
+  </si>
+  <si>
+    <t>IWm 05 a Schwere Hochlochziegel-Wohnungstrennwand</t>
+  </si>
+  <si>
+    <t>Hol</t>
+  </si>
+  <si>
+    <t>Neubau Holzbauweise</t>
+  </si>
+  <si>
+    <t>AWh02_Steinwolle</t>
+  </si>
+  <si>
+    <t>DAh 02a_Steinwolle</t>
+  </si>
+  <si>
+    <t>GDh 02 a</t>
+  </si>
+  <si>
+    <t>DAh 04a Terrasse</t>
+  </si>
+  <si>
+    <t>KDh 01 a</t>
+  </si>
+  <si>
+    <t>ADh 01 a Massivholzdecke über Außenluft, Nassestrich</t>
+  </si>
+  <si>
+    <t>IWh 02 a</t>
+  </si>
+  <si>
+    <t>Lei</t>
+  </si>
+  <si>
     <t>Neubau Leichtbau</t>
   </si>
   <si>
-    <t>Lei</t>
-  </si>
-  <si>
-    <t>Passivhaus</t>
-  </si>
-  <si>
     <t>AWl 01 a Holzständer-Außenwand, hinterlüftet</t>
   </si>
   <si>
     <t>DAl 05 a Doppel-T-Träger-Flachdach</t>
   </si>
   <si>
-    <t>Efo 01 a Plattenfundament, oberseitig gedämmt, Nassestrich</t>
-  </si>
-  <si>
     <t>GDl 01 a Leichtbau- (oder Tram-) Geschoßdecke, Nassestrich</t>
   </si>
   <si>
@@ -15737,103 +15833,7 @@
     <t>ADl 01 a</t>
   </si>
   <si>
-    <t>EAm 02 a Erdberührte Stahlbeton-Außenwand</t>
-  </si>
-  <si>
-    <t>IWl 01 a Ständer-Scheidewand, nichttragend</t>
-  </si>
-  <si>
     <t>IWl 04 a Leichtbau-Wohnungstrennwand, tragend</t>
-  </si>
-  <si>
-    <t>Erdberührte Wand Keller</t>
-  </si>
-  <si>
-    <t>1_UG_TG_BP_01d Bodenplatte STB 120 kg/m³ WU Beton bei drückendem Wasser, weiße Wanne, Asphaltbelag</t>
-  </si>
-  <si>
-    <t>1_UG_TG_Stü_01 Stützen</t>
-  </si>
-  <si>
-    <t>1_UG_TG_TW_01 Trennwand zu TG STB 100kg/m³ TG (tragend + Brandschutz)</t>
-  </si>
-  <si>
-    <t>Holz-Alu-Rahmen Fichte &gt;= 91 Stockrahmentiefe &lt; 109</t>
-  </si>
-  <si>
-    <t>Dreifach-Wärmeschutzglas, Argon, 40 &lt; Scheibenstärke</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>Bet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Neubau konventionell Stahlbeton </t>
-  </si>
-  <si>
-    <t>AWm 01 a Stahlbeton-Außenwand, WDVS</t>
-  </si>
-  <si>
-    <t>DAm 03 a Stahlbeton-Flachdach als Warmdach</t>
-  </si>
-  <si>
-    <t>GDm 01 a Stahlbeton-Geschoßdecke, Nassestrich (Nassräume)</t>
-  </si>
-  <si>
-    <t>DAm 06 a Stahlbeton-Flachdach mit Terrassenaufbau</t>
-  </si>
-  <si>
-    <t>KDu 01 a Kellerdecke massiv, unterseitig gedämmt</t>
-  </si>
-  <si>
-    <t>ADm 01 a Stahlbetondecke über Außenluft, Distanzboden</t>
-  </si>
-  <si>
-    <t>Neubau_Stb_IWm 05 a Schwere Hochlochziegel-Wohnungstrennwand</t>
-  </si>
-  <si>
-    <t>Zie</t>
-  </si>
-  <si>
-    <t>Neubau konventionell Ziegel</t>
-  </si>
-  <si>
-    <t>AWm 06 a Schwere Hochlochziegel-Außenwand, Spezial-WDVS</t>
-  </si>
-  <si>
-    <t>GDm 03 a Ziegel-Geschoßdecke ohne Aufbeton</t>
-  </si>
-  <si>
-    <t>IWm 05 a Schwere Hochlochziegel-Wohnungstrennwand</t>
-  </si>
-  <si>
-    <t>Hol</t>
-  </si>
-  <si>
-    <t>Neubau Holzbauweise</t>
-  </si>
-  <si>
-    <t>AWh02_Steinwolle</t>
-  </si>
-  <si>
-    <t>DAh 02a_Steinwolle</t>
-  </si>
-  <si>
-    <t>GDh 02 a</t>
-  </si>
-  <si>
-    <t>DAh 04a Terrasse</t>
-  </si>
-  <si>
-    <t>KDh 01 a</t>
-  </si>
-  <si>
-    <t>ADh 01 a Massivholzdecke über Außenluft, Nassestrich</t>
-  </si>
-  <si>
-    <t>IWh 02 a</t>
   </si>
   <si>
     <t>Hyb</t>
@@ -17173,70 +17173,8 @@
 </a:theme>
 </file>
 
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="8">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="0" width="0" row="0">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{689C6868-F4CC-41DD-81A9-29460501981F}">
-  <we:reference id="wa200006518" version="1.1.1.0" store="de-DE" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="wa200006518" version="1.1.1.0" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="pyscriptSettings" value="&quot;{\&quot;defaultMode\&quot;:2,\&quot;pyodideVersion\&quot;:\&quot;0.26.2\&quot;,\&quot;pyodidePackages\&quot;:[\&quot;numpy\&quot;,\&quot;pandas\&quot;,\&quot;matplotlib\&quot;,\&quot;statsmodels\&quot;],\&quot;pyscriptApps\&quot;:[],\&quot;micropipPackages\&quot;:[\&quot;seaborn==0.13.2\&quot;],\&quot;initCode\&quot;:\&quot;# Add imports\\nimport math\\nimport numpy as np\\nimport pandas as pd\\n\\n# Define classes and functions\\ndef to_df(data) -&gt; pd.DataFrame:\\n    \\\&quot;\\\&quot;\\\&quot;\\n    Converts a REF (i.e. list of lists) into a pandas DataFrame\\n    Assumes that the first row contains column headers\\n\\n    Usage: df = to_df(REF(\\\&quot;F15:H22\\\&quot;))\\n    \\\&quot;\\\&quot;\\\&quot;\\n    if isinstance(data, pd.DataFrame):\\n        return data\\n    if hasattr(data, '__len__') and len(data) &gt; 0 and hasattr(data[0], '__len__'):\\n        return pd.DataFrame(data[1:], columns=data[0])\\n    raise TypeError('Expected list of lists')\\n\\ndef to_array(data) -&gt; np.ndarray:\\n    \\\&quot;\\\&quot;\\\&quot;\\n    Converts a REF (i.e. list of lists) into a 2-dimensional numpy array\\n\\n    Usage: arr = to_array(REF(\\\&quot;B3:C44\\\&quot;))\\n    \\\&quot;\\\&quot;\\\&quot;\\n    if isinstance(data, np.ndarray):\\n        return data\\n    return np.array(data)\\n\\ndef to_list(data) -&gt; list:\\n    \\\&quot;\\\&quot;\\\&quot;\\n    Converts a REF (i.e. list of lists) into a 1-d list.\\n    Handles wide (1xn) or tall (nx1) data.\\n\\n    Usage: x = to_list(REF(\\\&quot;G1:G55\\\&quot;))\\n    \\\&quot;\\\&quot;\\\&quot;\\n    if not hasattr(data, '__len__'): # data is scalar\\n        return [data]\\n    if len(data) == 0 or not hasattr(data[0], '__len__'): # data is already a list\\n        return list(data)\\n    if len(data) == 1: # data is wide\\n        return list(data[0])\\n    elif len(data[0]) == 1: #data is tall\\n        return [x[0] for x in data]\\n    else:\\n        raise TypeError(f\\\&quot;data must be 1xn or nx1, not {len(data)}x{len(data[0])}\\\&quot;)\\n\\n\&quot;}&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-  <we:extLst>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
-      <we:containsCustomFunctions/>
-    </a:ext>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
-      <we:customFunctionIdList>
-        <we:customFunctionIds>_xldudf_PYSCRIPT_CODE</we:customFunctionIds>
-        <we:customFunctionIds>_xldudf_ANACONDA_CODE</we:customFunctionIds>
-      </we:customFunctionIdList>
-    </a:ext>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{0858819E-0033-43BF-8937-05EC82904868}">
-      <we:backgroundApp state="0" runtimeId="PyScript.Url"/>
-    </a:ext>
-  </we:extLst>
-</we:webextension>
-</file>
-
-<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{B6A2E36A-36CA-49EC-BD9E-E2D152C46B0D}">
-  <we:reference id="wa200007447" version="1.0.0.0" store="de-DE" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="WA200007447" version="1.0.0.0" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties/>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-  <we:extLst>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
-      <we:containsCustomFunctions/>
-    </a:ext>
-    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
-      <we:customFunctionIdList>
-        <we:customFunctionIds>_xldudf_BOARDFLARE_RUNPY</we:customFunctionIds>
-        <we:customFunctionIds>_xldudf_BOARDFLARE_EXEC</we:customFunctionIds>
-      </we:customFunctionIdList>
-    </a:ext>
-  </we:extLst>
-</we:webextension>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E8739E-8220-4FD6-913B-1FED19A49271}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A929CA-2448-4821-B638-FC1C32FA958F}">
   <sheetPr codeName="Tabelle2"/>
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -17286,7 +17224,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="1">
-        <v>46319.810150462959</v>
+        <v>46323.964594907404</v>
       </c>
     </row>
   </sheetData>
@@ -17295,7 +17233,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AC7E610-38FA-46D5-A63F-0228974C6AD8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91E6C12C-8FB3-4C53-AD54-B42697B04666}">
   <sheetPr codeName="Tabelle11"/>
   <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -17396,7 +17334,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1543A306-3AAD-49AC-B432-05EC04E1281C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D95C20A7-93AE-4AE3-A361-A3CA48206C48}">
   <sheetPr codeName="Tabelle12"/>
   <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -17479,7 +17417,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE326116-708F-4948-9249-80EA659174AE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7E10B80-5ECE-4DA5-ABF2-B5EAEEABE5DD}">
   <sheetPr codeName="Tabelle13"/>
   <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -17799,7 +17737,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8C378A0-1CD8-45F2-A0C6-7477E4233859}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A5986D1-1583-4403-8636-4F1D7995B2A6}">
   <sheetPr codeName="Tabelle14"/>
   <dimension ref="A1:M22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -18588,7 +18526,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26A511C6-992C-4874-9683-80C4984FC40C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C9ADB1-F056-4C47-A4F1-F2D6D092A7D4}">
   <sheetPr codeName="Tabelle15"/>
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -18943,7 +18881,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBF21AC7-311E-4547-BEAE-37CFAE1EF633}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D19AA2A2-164C-4A2A-BDB3-247FAFF4A3B4}">
   <sheetPr codeName="Tabelle16"/>
   <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -19068,7 +19006,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D09BB551-25C0-404D-BF64-4ADBBE079E47}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B137D2E-15B1-47B6-959E-64B6DC9386E0}">
   <sheetPr codeName="Tabelle17"/>
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -19414,7 +19352,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DF25DF9-B7A3-4F77-A4FD-4E9E044C3E07}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0B66374-89F6-463D-8BDD-1D88A22AFAFE}">
   <sheetPr codeName="Tabelle18"/>
   <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -19922,7 +19860,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{613BD04A-92AB-429D-901F-EB33635B1214}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82F70884-A59A-49C3-B1CE-5A6C37CFA07A}">
   <sheetPr codeName="Tabelle19"/>
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -20123,7 +20061,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAE9C9A8-8CF2-4BC0-8EBF-0F8B9F3D318A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB08D671-D2A7-4D96-A86D-A776543C8564}">
   <sheetPr codeName="Tabelle20"/>
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -20320,7 +20258,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB8B744-B063-41B5-A1A1-03CF23F94C97}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F813358C-23A9-4AFB-B138-6F7D0955931E}">
   <sheetPr codeName="Tabelle3"/>
   <dimension ref="A1:M799"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -42592,7 +42530,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64F679D0-FF54-4E7C-866C-FB820CA82803}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11359F6F-6456-4A74-A2D9-81E94B2C29F6}">
   <sheetPr codeName="Tabelle21"/>
   <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -43355,7 +43293,7 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57BAD9DC-6B31-4B9F-A59B-440271CCB966}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E217FCDC-FF45-4F76-8167-C870433712F2}">
   <sheetPr codeName="Tabelle22"/>
   <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -43900,7 +43838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB81B787-5841-4DBF-B5A0-019E7069C1C9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9871F036-FF67-40B3-B2EA-32F9449348F5}">
   <sheetPr codeName="Tabelle23"/>
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -44104,7 +44042,7 @@
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{478EA845-58C0-4000-B5B8-F10A64513141}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D109601-1E17-43A0-BB30-677EC1028D5D}">
   <sheetPr codeName="Tabelle24"/>
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -44308,7 +44246,7 @@
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C9D0D8C-AE62-4AE1-B87D-A498E9325696}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E952F8A1-5A88-4219-A184-27730684B1F1}">
   <sheetPr codeName="Tabelle25"/>
   <dimension ref="A1:S6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -44609,7 +44547,7 @@
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84397217-F489-46AE-A322-0CC8D83599FA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{751BBC54-93E6-482E-9DFC-476E5948C80D}">
   <sheetPr codeName="Tabelle26"/>
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -44742,13 +44680,13 @@
         <v>692</v>
       </c>
       <c r="D8">
-        <v>128.94</v>
+        <v>8.0324999999999971</v>
       </c>
       <c r="F8">
-        <v>128.94</v>
+        <v>8.0324999999999971</v>
       </c>
       <c r="G8">
-        <v>257.88</v>
+        <v>16.064999999999994</v>
       </c>
     </row>
   </sheetData>
@@ -44757,7 +44695,7 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0BA5500-4481-470D-A123-ED99CFCD2535}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C258E6E-2300-4730-A4CB-D0C47DA283A1}">
   <sheetPr codeName="Tabelle27"/>
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -44912,7 +44850,7 @@
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F7E0A3-B718-4F09-B7CB-68AAE0E5BA6B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE566258-8EC0-4C67-93D7-6CD38CF1083B}">
   <sheetPr codeName="Tabelle28"/>
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -45072,7 +45010,7 @@
 </file>
 
 <file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90BB12A5-F73F-45AE-AB1E-317AABEA1866}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A38C202-AA60-4E81-B6D5-3EBF5C79BD68}">
   <sheetPr codeName="Tabelle29"/>
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -45272,7 +45210,7 @@
 </file>
 
 <file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB95A3EB-FCFF-47B3-B012-AF9B71E4D43F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34299757-8ABC-43BA-A7A5-2B5B8D348C65}">
   <sheetPr codeName="Tabelle30"/>
   <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -45427,7 +45365,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E129EDB-AB2D-4094-BD47-7643CA091173}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0865F008-896A-4112-8119-F03DA3DDCCC1}">
   <sheetPr codeName="Tabelle4"/>
   <dimension ref="A1:M618"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -47057,7 +46995,7 @@
         <v>3052</v>
       </c>
       <c r="K54" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M54" s="6" t="s">
         <v>3543</v>
@@ -47577,7 +47515,7 @@
         <v>3054</v>
       </c>
       <c r="K71" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M71" s="6" t="s">
         <v>3560</v>
@@ -52781,7 +52719,7 @@
         <v>3171</v>
       </c>
       <c r="K245" s="5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M245" s="6" t="s">
         <v>3716</v>
@@ -61257,7 +61195,7 @@
 </file>
 
 <file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1FB1F0C-6E1A-4FB7-A4FD-7D69DC3F9EFA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F730113-C496-42B0-8622-191B4893BC45}">
   <sheetPr codeName="Tabelle31"/>
   <dimension ref="A1:AB36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -61291,16 +61229,16 @@
         <v>5224</v>
       </c>
       <c r="G1" t="s">
+        <v>5206</v>
+      </c>
+      <c r="H1" t="s">
         <v>5225</v>
       </c>
-      <c r="H1" t="s">
-        <v>5234</v>
-      </c>
       <c r="I1" t="s">
+        <v>5230</v>
+      </c>
+      <c r="J1" t="s">
         <v>5239</v>
-      </c>
-      <c r="J1" t="s">
-        <v>5206</v>
       </c>
       <c r="K1" t="s">
         <v>5248</v>
@@ -61371,16 +61309,16 @@
         <v>4916</v>
       </c>
       <c r="G2" t="s">
+        <v>5205</v>
+      </c>
+      <c r="H2" t="s">
         <v>5226</v>
       </c>
-      <c r="H2" t="s">
-        <v>5235</v>
-      </c>
       <c r="I2" t="s">
+        <v>5231</v>
+      </c>
+      <c r="J2" t="s">
         <v>5240</v>
-      </c>
-      <c r="J2" t="s">
-        <v>5205</v>
       </c>
       <c r="K2" t="s">
         <v>5249</v>
@@ -61445,16 +61383,16 @@
         <v>5205</v>
       </c>
       <c r="G3" t="s">
+        <v>5205</v>
+      </c>
+      <c r="H3" t="s">
         <v>5226</v>
       </c>
-      <c r="H3" t="s">
-        <v>5235</v>
-      </c>
       <c r="I3" t="s">
+        <v>5231</v>
+      </c>
+      <c r="J3" t="s">
         <v>5240</v>
-      </c>
-      <c r="J3" t="s">
-        <v>5205</v>
       </c>
       <c r="K3" t="s">
         <v>5249</v>
@@ -61519,16 +61457,16 @@
         <v>5206</v>
       </c>
       <c r="G4" t="s">
+        <v>5206</v>
+      </c>
+      <c r="H4" t="s">
         <v>5225</v>
       </c>
-      <c r="H4" t="s">
-        <v>5234</v>
-      </c>
       <c r="I4" t="s">
+        <v>5230</v>
+      </c>
+      <c r="J4" t="s">
         <v>5239</v>
-      </c>
-      <c r="J4" t="s">
-        <v>5206</v>
       </c>
       <c r="K4" t="s">
         <v>5248</v>
@@ -61753,16 +61691,16 @@
         <v>5208</v>
       </c>
       <c r="G10" t="s">
+        <v>5208</v>
+      </c>
+      <c r="H10" t="s">
         <v>5227</v>
       </c>
-      <c r="H10" t="s">
-        <v>5236</v>
-      </c>
       <c r="I10" t="s">
+        <v>5232</v>
+      </c>
+      <c r="J10" t="s">
         <v>5241</v>
-      </c>
-      <c r="J10" t="s">
-        <v>5208</v>
       </c>
       <c r="K10" t="s">
         <v>5250</v>
@@ -61838,19 +61776,19 @@
         <v>5209</v>
       </c>
       <c r="G12" t="s">
-        <v>5228</v>
+        <v>5209</v>
       </c>
       <c r="H12" t="s">
-        <v>5228</v>
+        <v>5209</v>
       </c>
       <c r="I12" t="s">
+        <v>5233</v>
+      </c>
+      <c r="J12" t="s">
         <v>5242</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>5209</v>
-      </c>
-      <c r="K12" t="s">
-        <v>5228</v>
       </c>
       <c r="L12" t="s">
         <v>5254</v>
@@ -61997,25 +61935,25 @@
         <v>5211</v>
       </c>
       <c r="G15" t="s">
-        <v>5229</v>
+        <v>5211</v>
       </c>
       <c r="H15" t="s">
-        <v>5237</v>
+        <v>5228</v>
       </c>
       <c r="I15" t="s">
+        <v>5234</v>
+      </c>
+      <c r="J15" t="s">
         <v>5243</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>5211</v>
-      </c>
-      <c r="K15" t="s">
-        <v>5229</v>
       </c>
       <c r="L15" t="s">
         <v>5256</v>
       </c>
       <c r="M15" t="s">
-        <v>5237</v>
+        <v>5228</v>
       </c>
       <c r="N15" t="s">
         <v>5272</v>
@@ -62041,19 +61979,19 @@
         <v>5212</v>
       </c>
       <c r="G16" t="s">
-        <v>5230</v>
+        <v>5212</v>
       </c>
       <c r="H16" t="s">
-        <v>5230</v>
+        <v>5212</v>
       </c>
       <c r="I16" t="s">
+        <v>5235</v>
+      </c>
+      <c r="J16" t="s">
         <v>5244</v>
       </c>
-      <c r="J16" t="s">
+      <c r="K16" t="s">
         <v>5212</v>
-      </c>
-      <c r="K16" t="s">
-        <v>5230</v>
       </c>
       <c r="L16" t="s">
         <v>5257</v>
@@ -62085,19 +62023,19 @@
         <v>5213</v>
       </c>
       <c r="G17" t="s">
-        <v>5231</v>
+        <v>5213</v>
       </c>
       <c r="H17" t="s">
-        <v>5231</v>
+        <v>5213</v>
       </c>
       <c r="I17" t="s">
+        <v>5236</v>
+      </c>
+      <c r="J17" t="s">
         <v>5245</v>
       </c>
-      <c r="J17" t="s">
+      <c r="K17" t="s">
         <v>5213</v>
-      </c>
-      <c r="K17" t="s">
-        <v>5231</v>
       </c>
       <c r="L17" t="s">
         <v>5258</v>
@@ -62170,19 +62108,19 @@
         <v>5214</v>
       </c>
       <c r="G19" t="s">
-        <v>5232</v>
+        <v>5214</v>
       </c>
       <c r="H19" t="s">
-        <v>5232</v>
+        <v>5214</v>
       </c>
       <c r="I19" t="s">
+        <v>5237</v>
+      </c>
+      <c r="J19" t="s">
         <v>5246</v>
       </c>
-      <c r="J19" t="s">
+      <c r="K19" t="s">
         <v>5214</v>
-      </c>
-      <c r="K19" t="s">
-        <v>5232</v>
       </c>
       <c r="L19" t="s">
         <v>5259</v>
@@ -62318,19 +62256,19 @@
         <v>5216</v>
       </c>
       <c r="G21" t="s">
-        <v>5233</v>
+        <v>5217</v>
       </c>
       <c r="H21" t="s">
+        <v>5229</v>
+      </c>
+      <c r="I21" t="s">
         <v>5238</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>5247</v>
       </c>
-      <c r="J21" t="s">
+      <c r="K21" t="s">
         <v>5217</v>
-      </c>
-      <c r="K21" t="s">
-        <v>5233</v>
       </c>
       <c r="L21" t="s">
         <v>5261</v>
@@ -62377,7 +62315,7 @@
         <v>5216</v>
       </c>
       <c r="L22" t="s">
-        <v>5233</v>
+        <v>5217</v>
       </c>
       <c r="M22" t="s">
         <v>5267</v>
@@ -62831,7 +62769,7 @@
 </file>
 
 <file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93F98929-14E2-42A3-907D-F97067CF1C6F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1C15181-609F-4F06-8CCE-D0DEB4D6CCA2}">
   <sheetPr codeName="Tabelle32"/>
   <dimension ref="A1:CU51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -71380,7 +71318,7 @@
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2">
-        <v>4136</v>
+        <v>123.17571</v>
       </c>
       <c r="F30" s="2">
         <v>147.67714282119744</v>
@@ -71974,7 +71912,7 @@
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2">
-        <v>2149</v>
+        <v>133.87499999999997</v>
       </c>
       <c r="F32" s="2">
         <v>171.48</v>
@@ -72568,7 +72506,7 @@
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2">
-        <v>2149</v>
+        <v>133.87499999999997</v>
       </c>
       <c r="F34" s="2">
         <v>0</v>
@@ -72865,7 +72803,7 @@
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2">
-        <v>8550.4</v>
+        <v>0</v>
       </c>
       <c r="F35" s="2">
         <v>0</v>
@@ -77320,7 +77258,7 @@
       </c>
       <c r="D50" s="2"/>
       <c r="E50" s="2">
-        <v>828.00000000000011</v>
+        <v>6.5210669999999995</v>
       </c>
       <c r="F50" s="2">
         <v>0</v>
@@ -77617,7 +77555,7 @@
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2">
-        <v>1931.9999999999998</v>
+        <v>15.215822999999995</v>
       </c>
       <c r="F51" s="2">
         <v>0</v>
@@ -77908,7 +77846,7 @@
 </file>
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B62BA44-1A9F-4EFB-992F-906979FBB894}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBBC8494-990D-4BAC-9056-47433897695C}">
   <sheetPr codeName="Tabelle33"/>
   <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -77990,7 +77928,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D7CDB55-FF3C-4D3E-938F-5022909E20CB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7789EC4A-1CB5-4B96-8EAE-553E3D323FFA}">
   <sheetPr codeName="Tabelle5"/>
   <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -79340,7 +79278,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D003A76F-6998-47F3-BE16-91FE7BFA535A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F895E754-E4E5-4EE6-9CDE-4810C20743A4}">
   <sheetPr codeName="Tabelle6"/>
   <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -79469,7 +79407,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61415428-6F90-4E8B-8689-2DC8429A1002}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{014308F7-3A24-4AC9-91CA-1B84CA1FFBCC}">
   <sheetPr codeName="Tabelle7"/>
   <dimension ref="A1:E402"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -85732,7 +85670,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A5B51FB-94A9-45EC-AE74-B6B7931A69E5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49952B5D-AC6F-45FB-8E9C-B36590061AFA}">
   <sheetPr codeName="Tabelle8"/>
   <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -86030,7 +85968,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C5F513F-E730-4088-93D7-2267807C58D0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8986D162-DB57-4433-B253-8FF691FC41A0}">
   <sheetPr codeName="Tabelle9"/>
   <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -87570,7 +87508,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E51BFBF5-DE4E-4D9C-8ED5-BECD817C4D35}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A8208CB-A56E-4B8F-8422-C2DE1EE63BAC}">
   <sheetPr codeName="Tabelle10"/>
   <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>